<commit_message>
Fix RAB rebar formula, lean support-building prices; verify formulas
Rebar quantity referenced the Rupiah column instead of volume. Support
building unit prices lowered to semi-permanent levels. Formulas checked with
a Python evaluator (0 errors); LibreOffice recalculation is unavailable here,
so cached values are empty until opened in Excel.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Rt4P5tNoMcDQDdSmTGefKt
</commit_message>
<xml_diff>
--- a/kandang-kub-2000/RAB-Kandang-Ayam-KUB-2000-Ekor-Konawe-Selatan.xlsx
+++ b/kandang-kub-2000/RAB-Kandang-Ayam-KUB-2000-Ekor-Konawe-Selatan.xlsx
@@ -5946,7 +5946,7 @@
         </is>
       </c>
       <c r="C17" s="31">
-        <f>(F14+F15+F16)*Asumsi!$B$35</f>
+        <f>(C14+C15+C16)*Asumsi!$B$35</f>
         <v/>
       </c>
       <c r="D17" s="27" t="inlineStr">
@@ -6696,7 +6696,7 @@
         </is>
       </c>
       <c r="E6" s="21" t="n">
-        <v>2800000</v>
+        <v>1800000</v>
       </c>
       <c r="F6" s="12">
         <f>ROUND(C6*E6,0)</f>
@@ -6704,7 +6704,7 @@
       </c>
       <c r="G6" s="32" t="inlineStr">
         <is>
-          <t>Bata setengah, rangka baja ringan, lantai beton, anti tikus.</t>
+          <t>Semi-permanen: bata setengah, rangka atap sederhana, lantai beton, anti tikus.</t>
         </is>
       </c>
     </row>
@@ -6726,7 +6726,7 @@
         </is>
       </c>
       <c r="E7" s="21" t="n">
-        <v>2800000</v>
+        <v>2000000</v>
       </c>
       <c r="F7" s="12">
         <f>ROUND(C7*E7,0)</f>
@@ -6734,7 +6734,7 @@
       </c>
       <c r="G7" s="32" t="inlineStr">
         <is>
-          <t>Sejuk, berventilasi, lantai keramik atau plester halus.</t>
+          <t>Sejuk, berventilasi, lantai plester halus.</t>
         </is>
       </c>
     </row>
@@ -6756,7 +6756,7 @@
         </is>
       </c>
       <c r="E8" s="21" t="n">
-        <v>3000000</v>
+        <v>2200000</v>
       </c>
       <c r="F8" s="12">
         <f>ROUND(C8*E8,0)</f>
@@ -6764,7 +6764,7 @@
       </c>
       <c r="G8" s="32" t="inlineStr">
         <is>
-          <t>Termasuk ruang ganti dan kamar mandi sederhana.</t>
+          <t>Termasuk kamar mandi sederhana.</t>
         </is>
       </c>
     </row>
@@ -6786,7 +6786,7 @@
         </is>
       </c>
       <c r="E9" s="21" t="n">
-        <v>2000000</v>
+        <v>1500000</v>
       </c>
       <c r="F9" s="12">
         <f>ROUND(C9*E9,0)</f>
@@ -6816,7 +6816,7 @@
         </is>
       </c>
       <c r="E10" s="21" t="n">
-        <v>750000</v>
+        <v>500000</v>
       </c>
       <c r="F10" s="12">
         <f>ROUND(C10*E10,0)</f>
@@ -6847,7 +6847,7 @@
         </is>
       </c>
       <c r="E11" s="21" t="n">
-        <v>175000</v>
+        <v>120000</v>
       </c>
       <c r="F11" s="12">
         <f>ROUND(C11*E11,0)</f>
@@ -6855,7 +6855,7 @@
       </c>
       <c r="G11" s="32" t="inlineStr">
         <is>
-          <t>Kawat harmonika + tiang beton tiap 2,5 m.</t>
+          <t>Kawat harmonika + tiang beton/kayu tiap 2,5 m.</t>
         </is>
       </c>
     </row>

</xml_diff>